<commit_message>
Semente: os 35 materiais nunca comprados ganham referência de mercado em SP
Preços pesquisados em set/2026 — SINAPI-SP jul/2026 (buscadorsinapi.com.br)
para disjuntores tripolares, conjuntos de interruptores e tomadas, placas,
caixa octogonal; varejo de SP (Leroy Merlin, Telhanorte, Dimensional, ABC
Transformadores) para aquecedor a gás e kit de instalação, luminárias e
lâmpadas LED, refletores, balizadores, anel de vedação, caixa de inspeção
60x60, eletroduto 3", caixas de passagem metálicas, barramento. Fonte e
produto ficam na observação de cada insumo; precoFonte "mercado",
precoData 2026-09-06. Transformador: preço de compra (não há locação
publicada), marcado na observação. Nenhum material da semente fica sem
preço (917 insumos).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SiiMYe4saTp6wrW4PdVqhW
</commit_message>
<xml_diff>
--- a/docs/referencia-orcamento/SEMENTE-CADASTRO-REVISAO.xlsx
+++ b/docs/referencia-orcamento/SEMENTE-CADASTRO-REVISAO.xlsx
@@ -36,7 +36,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +58,11 @@
         <fgColor rgb="00FFF3C4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DFF5E1"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -71,13 +76,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -737,20 +743,34 @@
           <t>(kit)</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="n"/>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>2650</v>
+      </c>
       <c r="F7" s="3" t="n"/>
-      <c r="G7" s="2" t="n"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Aquecedor a gás Rinnai E21 21 L/min GLP digital</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Leroy Merlin: https://www.leroymerlin.com.br/aquecedor-de-agua-a-gas-rinnai-21l-min-glp-branco-digital-e21_89839351</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -768,20 +788,34 @@
           <t>(kit)</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="n"/>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>464.8</v>
+      </c>
       <c r="F8" s="3" t="n"/>
-      <c r="G8" s="2" t="n"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Kit instalação Lorenzetti (flexíveis + registro de gás) R$ 279,90 + kit exaustão 80 mm x 1,5 m WDB R$ 184,90</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Telhanorte: https://www.telhanorte.com.br/kit-de-instalacao-de-aquecedor-de-agua-a-gas-lorenzetti-1587897/p | soma de dois kits; versão econômica dos flexíveis: R$ 349,80 no total</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3275,20 +3309,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D69" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E69" s="3" t="n"/>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="n">
+        <v>245.7</v>
+      </c>
       <c r="F69" s="3" t="n"/>
-      <c r="G69" s="2" t="n"/>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H69" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I69" s="2" t="n"/>
-      <c r="J69" s="2" t="inlineStr"/>
-      <c r="K69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>3 × barramento pente trifásico 12 polos 80A Steck (R$ 81,90 cada)</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>Telhanorte: https://www.telhanorte.com.br/barramento-trifasico-80a-220440v-3x4p-din-steck-980366/p | não há pente 100A/32 disj. no varejo consultado; 3 pentes de 12 polos 80A cobrem 32 disjuntores</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4376,20 +4424,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D96" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E96" s="3" t="n"/>
+      <c r="D96" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="n">
+        <v>322.39</v>
+      </c>
       <c r="F96" s="3" t="n"/>
-      <c r="G96" s="2" t="n"/>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H96" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I96" s="2" t="n"/>
-      <c r="J96" s="2" t="inlineStr"/>
-      <c r="K96" s="2" t="inlineStr"/>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP insumo 2391 — disjuntor termomagnético tripolar 125A</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP jul/2026: https://buscadorsinapi.com.br/sp/insumo/2391</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -4530,20 +4592,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D100" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E100" s="3" t="n"/>
+      <c r="D100" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="n">
+        <v>59.1</v>
+      </c>
       <c r="F100" s="3" t="n"/>
-      <c r="G100" s="2" t="n"/>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H100" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I100" s="2" t="n"/>
-      <c r="J100" s="2" t="inlineStr"/>
-      <c r="K100" s="2" t="inlineStr"/>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP insumo 34709 — disjuntor DIN tripolar 10–50A</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP jul/2026: https://buscadorsinapi.com.br/sp/insumo/34709</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -4602,20 +4678,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D102" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E102" s="3" t="n"/>
+      <c r="D102" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="n">
+        <v>259.9</v>
+      </c>
       <c r="F102" s="3" t="n"/>
-      <c r="G102" s="2" t="n"/>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H102" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I102" s="2" t="n"/>
-      <c r="J102" s="2" t="inlineStr"/>
-      <c r="K102" s="2" t="inlineStr"/>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>Disjuntor tripolar 80A curva C 10kA Steck</t>
+        </is>
+      </c>
+      <c r="K102" s="2" t="inlineStr">
+        <is>
+          <t>Telhanorte: https://www.telhanorte.com.br/disjuntor-tripolar-80a-curva-c-steck-1399640/p | SINAPI-SP 2373 (NEMA 60–100A) = R$ 103,09 como referência inferior</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -5043,20 +5133,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D113" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E113" s="3" t="n"/>
+      <c r="D113" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="n">
+        <v>70.59</v>
+      </c>
       <c r="F113" s="3" t="n"/>
-      <c r="G113" s="2" t="n"/>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H113" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I113" s="2" t="n"/>
-      <c r="J113" s="2" t="inlineStr"/>
-      <c r="K113" s="2" t="inlineStr"/>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP insumo 34714 — disjuntor DIN tripolar 63A</t>
+        </is>
+      </c>
+      <c r="K113" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP jul/2026: https://buscadorsinapi.com.br/sp/insumo/34714 | insumo SINAPI não especifica 10kA</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -5103,7 +5207,7 @@
       </c>
       <c r="K114" s="2" t="inlineStr">
         <is>
-          <t>preço herdado de 'Elétrica - Disjuntor Bipolar 10A - 10kA' por similaridade (0.67)</t>
+          <t>preço herdado de 'Elétrica - Disjuntor Bipolar 10A - 10kA' por similaridade (0.67) — conferir</t>
         </is>
       </c>
     </row>
@@ -5496,20 +5600,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D124" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E124" s="3" t="n"/>
+      <c r="D124" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="n">
+        <v>25.1</v>
+      </c>
       <c r="F124" s="3" t="n"/>
-      <c r="G124" s="2" t="n"/>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H124" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I124" s="2" t="n"/>
-      <c r="J124" s="2" t="inlineStr"/>
-      <c r="K124" s="2" t="inlineStr"/>
+      <c r="J124" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP insumo 38073 — 1 simples + 2 paralelos, conjunto 4x2 com placa</t>
+        </is>
+      </c>
+      <c r="K124" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP jul/2026: https://buscadorsinapi.com.br/sp/insumo/38073</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -5527,20 +5645,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D125" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E125" s="3" t="n"/>
+      <c r="D125" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="n">
+        <v>22.6</v>
+      </c>
       <c r="F125" s="3" t="n"/>
-      <c r="G125" s="2" t="n"/>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H125" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I125" s="2" t="n"/>
-      <c r="J125" s="2" t="inlineStr"/>
-      <c r="K125" s="2" t="inlineStr"/>
+      <c r="J125" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP insumo 38072 — 2 simples + 1 paralelo, conjunto 4x2 com placa</t>
+        </is>
+      </c>
+      <c r="K125" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP jul/2026: https://buscadorsinapi.com.br/sp/insumo/38072</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -5558,20 +5690,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D126" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E126" s="3" t="n"/>
+      <c r="D126" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E126" s="3" t="n">
+        <v>18.65</v>
+      </c>
       <c r="F126" s="3" t="n"/>
-      <c r="G126" s="2" t="n"/>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H126" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I126" s="2" t="n"/>
-      <c r="J126" s="2" t="inlineStr"/>
-      <c r="K126" s="2" t="inlineStr"/>
+      <c r="J126" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP insumo 38071 — 3 interruptores simples, conjunto 4x2 com placa</t>
+        </is>
+      </c>
+      <c r="K126" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP jul/2026: https://buscadorsinapi.com.br/sp/insumo/38071</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -5618,7 +5764,7 @@
       </c>
       <c r="K127" s="2" t="inlineStr">
         <is>
-          <t>preço herdado de 'Elétrica - Interruptores e placas - Interruptor paralela - 1 tecla' por similaridade (0.75)</t>
+          <t>preço herdado de 'Elétrica - Interruptores e placas - Interruptor paralela - 1 tecla' por similaridade (0.75) — conferir</t>
         </is>
       </c>
     </row>
@@ -5679,20 +5825,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D129" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E129" s="3" t="n"/>
+      <c r="D129" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="n">
+        <v>27.4</v>
+      </c>
       <c r="F129" s="3" t="n"/>
-      <c r="G129" s="2" t="n"/>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H129" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I129" s="2" t="n"/>
-      <c r="J129" s="2" t="inlineStr"/>
-      <c r="K129" s="2" t="inlineStr"/>
+      <c r="J129" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP insumo 38074 — 3 interruptores paralelos, conjunto 4x2 com placa</t>
+        </is>
+      </c>
+      <c r="K129" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP jul/2026: https://buscadorsinapi.com.br/sp/insumo/38074</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -5739,7 +5899,7 @@
       </c>
       <c r="K130" s="2" t="inlineStr">
         <is>
-          <t>preço herdado de 'Elétrica - Interruptores e placas - Interruptor simples e paralelo 2 teclas' por similaridade (0.88)</t>
+          <t>preço herdado de 'Elétrica - Interruptores e placas - Interruptor simples e paralelo 2 teclas' por similaridade (0.88) — conferir</t>
         </is>
       </c>
     </row>
@@ -5788,7 +5948,7 @@
       </c>
       <c r="K131" s="2" t="inlineStr">
         <is>
-          <t>preço herdado de 'Elétrica - Interruptores e placas - Interruptor paralela - 1 tecla' por similaridade (0.75)</t>
+          <t>preço herdado de 'Elétrica - Interruptores e placas - Interruptor paralela - 1 tecla' por similaridade (0.75) — conferir</t>
         </is>
       </c>
     </row>
@@ -5837,7 +5997,7 @@
       </c>
       <c r="K132" s="2" t="inlineStr">
         <is>
-          <t>preço herdado de 'Elétrica - Interruptores e placas - Interruptor simples e paralelo 2 teclas' por similaridade (0.88)</t>
+          <t>preço herdado de 'Elétrica - Interruptores e placas - Interruptor simples e paralelo 2 teclas' por similaridade (0.88) — conferir</t>
         </is>
       </c>
     </row>
@@ -5857,20 +6017,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D133" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E133" s="3" t="n"/>
+      <c r="D133" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="n">
+        <v>18.65</v>
+      </c>
       <c r="F133" s="3" t="n"/>
-      <c r="G133" s="2" t="n"/>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H133" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I133" s="2" t="n"/>
-      <c r="J133" s="2" t="inlineStr"/>
-      <c r="K133" s="2" t="inlineStr"/>
+      <c r="J133" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP insumo 38071 — 3 interruptores simples, conjunto 4x2 com placa</t>
+        </is>
+      </c>
+      <c r="K133" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP jul/2026: https://buscadorsinapi.com.br/sp/insumo/38071 | mesmo insumo de 'Interruptor 3 teclas simples' (nome duplicado no cadastro)</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -5970,20 +6144,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D136" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E136" s="3" t="n"/>
+      <c r="D136" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E136" s="3" t="n">
+        <v>8.19</v>
+      </c>
       <c r="F136" s="3" t="n"/>
-      <c r="G136" s="2" t="n"/>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H136" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I136" s="2" t="n"/>
-      <c r="J136" s="2" t="inlineStr"/>
-      <c r="K136" s="2" t="inlineStr"/>
+      <c r="J136" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP 38095 placa cega 4x4 (R$ 5,53) + 38100 suporte 4x4 (R$ 2,66)</t>
+        </is>
+      </c>
+      <c r="K136" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP jul/2026: https://buscadorsinapi.com.br/sp/insumo/38095</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -6083,20 +6271,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D139" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E139" s="3" t="n"/>
+      <c r="D139" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E139" s="3" t="n">
+        <v>4.1</v>
+      </c>
       <c r="F139" s="3" t="n"/>
-      <c r="G139" s="2" t="n"/>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H139" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I139" s="2" t="n"/>
-      <c r="J139" s="2" t="inlineStr"/>
-      <c r="K139" s="2" t="inlineStr"/>
+      <c r="J139" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP 38092 placa 4x2 1 posto (R$ 2,47) + 38099 suporte 4x2 (R$ 1,63)</t>
+        </is>
+      </c>
+      <c r="K139" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP jul/2026: https://buscadorsinapi.com.br/sp/insumo/38092</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -6114,20 +6316,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D140" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E140" s="3" t="n"/>
+      <c r="D140" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E140" s="3" t="n">
+        <v>4.1</v>
+      </c>
       <c r="F140" s="3" t="n"/>
-      <c r="G140" s="2" t="n"/>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H140" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I140" s="2" t="n"/>
-      <c r="J140" s="2" t="inlineStr"/>
-      <c r="K140" s="2" t="inlineStr"/>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>mesma referência da placa 4x2 1 posto + suporte (placa redonda não encontrada nas fontes de SP)</t>
+        </is>
+      </c>
+      <c r="K140" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP jul/2026: https://buscadorsinapi.com.br/sp/insumo/38092 | placa redonda de condulete costuma custar mais no varejo</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -6227,20 +6443,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D143" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E143" s="3" t="n"/>
+      <c r="D143" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E143" s="3" t="n">
+        <v>16.76</v>
+      </c>
       <c r="F143" s="3" t="n"/>
-      <c r="G143" s="2" t="n"/>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H143" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I143" s="2" t="n"/>
-      <c r="J143" s="2" t="inlineStr"/>
-      <c r="K143" s="2" t="inlineStr"/>
+      <c r="J143" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP insumo 38084 — tomada para antena de TV coaxial, conjunto 4x2 com placa</t>
+        </is>
+      </c>
+      <c r="K143" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP jul/2026: https://buscadorsinapi.com.br/sp/insumo/38084</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -6299,20 +6529,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D145" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E145" s="3" t="n"/>
+      <c r="D145" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E145" s="3" t="n">
+        <v>17.15</v>
+      </c>
       <c r="F145" s="3" t="n"/>
-      <c r="G145" s="2" t="n"/>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H145" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I145" s="2" t="n"/>
-      <c r="J145" s="2" t="inlineStr"/>
-      <c r="K145" s="2" t="inlineStr"/>
+      <c r="J145" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP insumo 38075 — tomada 2P+T 20A, conjunto 4x2 com placa e suporte</t>
+        </is>
+      </c>
+      <c r="K145" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP jul/2026: https://buscadorsinapi.com.br/sp/insumo/38075 | só o módulo (38102) = R$ 10,78</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -6494,20 +6738,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D150" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E150" s="3" t="n"/>
+      <c r="D150" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="n">
+        <v>159.9</v>
+      </c>
       <c r="F150" s="3" t="n"/>
-      <c r="G150" s="2" t="n"/>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H150" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I150" s="2" t="n"/>
-      <c r="J150" s="2" t="inlineStr"/>
-      <c r="K150" s="2" t="inlineStr"/>
+      <c r="J150" s="2" t="inlineStr">
+        <is>
+          <t>Luminária LED downlight embutir 25W Taschibra (equivalente; Ledvance 25W sem estoque em SP)</t>
+        </is>
+      </c>
+      <c r="K150" s="2" t="inlineStr">
+        <is>
+          <t>Leroy Merlin: https://www.leroymerlin.com.br/luminaria-de-teto-plafon-led-taschibra-downlight-max-25w-embutir-redondo-luz-fria-6500k_1571055158 | Ledvance 31W na Dimensional: R$ 208,99</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -6525,20 +6783,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D151" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E151" s="3" t="n"/>
+      <c r="D151" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="n">
+        <v>166.99</v>
+      </c>
       <c r="F151" s="3" t="n"/>
-      <c r="G151" s="2" t="n"/>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H151" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I151" s="2" t="n"/>
-      <c r="J151" s="2" t="inlineStr"/>
-      <c r="K151" s="2" t="inlineStr"/>
+      <c r="J151" s="2" t="inlineStr">
+        <is>
+          <t>Luminária LED redonda embutir Ledvance 35W 4000K (cód. 7014862)</t>
+        </is>
+      </c>
+      <c r="K151" s="2" t="inlineStr">
+        <is>
+          <t>Dimensional (SP): https://www.dimensional.com.br/luminaria-led-red-emb-br-biv-4000k-35w-7014862-ledvance/p</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -6556,20 +6828,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D152" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E152" s="3" t="n"/>
+      <c r="D152" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="n">
+        <v>37.99</v>
+      </c>
       <c r="F152" s="3" t="n"/>
-      <c r="G152" s="2" t="n"/>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H152" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I152" s="2" t="n"/>
-      <c r="J152" s="2" t="inlineStr"/>
-      <c r="K152" s="2" t="inlineStr"/>
+      <c r="J152" s="2" t="inlineStr">
+        <is>
+          <t>Painel LED quadrado embutir 18W Philips (equivalente; Ledvance 18W sem estoque)</t>
+        </is>
+      </c>
+      <c r="K152" s="2" t="inlineStr">
+        <is>
+          <t>Dimensional (SP): https://www.dimensional.com.br/luminaria-led-plafon-quad-emb-ac-br-ip20-biv-6500k-18w-angu-leddl252quadra---philips/p</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -7653,20 +7939,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D179" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E179" s="3" t="n"/>
+      <c r="D179" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E179" s="3" t="n">
+        <v>12.99</v>
+      </c>
       <c r="F179" s="3" t="n"/>
-      <c r="G179" s="2" t="n"/>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H179" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I179" s="2" t="n"/>
-      <c r="J179" s="2" t="inlineStr"/>
-      <c r="K179" s="2" t="inlineStr"/>
+      <c r="J179" s="2" t="inlineStr">
+        <is>
+          <t>Lâmpada LED PAR20 7W E27 Intral</t>
+        </is>
+      </c>
+      <c r="K179" s="2" t="inlineStr">
+        <is>
+          <t>Dimensional (SP): https://www.dimensional.com.br/lampada-led-par20-e27-6500k-biv-7w-525lm-36g-07564-intral/p</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -7684,20 +7984,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D180" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E180" s="3" t="n"/>
+      <c r="D180" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E180" s="3" t="n">
+        <v>10.9</v>
+      </c>
       <c r="F180" s="3" t="n"/>
-      <c r="G180" s="2" t="n"/>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H180" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I180" s="2" t="n"/>
-      <c r="J180" s="2" t="inlineStr"/>
-      <c r="K180" s="2" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr">
+        <is>
+          <t>Lâmpada LED PAR20 8W E27 Blumenau (9W indisponível)</t>
+        </is>
+      </c>
+      <c r="K180" s="2" t="inlineStr">
+        <is>
+          <t>Leroy Merlin: https://www.leroymerlin.com.br/lampada-led-blumenau-par20-8w-bivolt-3000k-e27-01071013_1572435564</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -7715,20 +8029,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D181" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E181" s="3" t="n"/>
+      <c r="D181" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E181" s="3" t="n">
+        <v>56.99</v>
+      </c>
       <c r="F181" s="3" t="n"/>
-      <c r="G181" s="2" t="n"/>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H181" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I181" s="2" t="n"/>
-      <c r="J181" s="2" t="inlineStr"/>
-      <c r="K181" s="2" t="inlineStr"/>
+      <c r="J181" s="2" t="inlineStr">
+        <is>
+          <t>Lâmpada LED PAR30 9,5W E27 Philips</t>
+        </is>
+      </c>
+      <c r="K181" s="2" t="inlineStr">
+        <is>
+          <t>Dimensional (SP): https://www.dimensional.com.br/lampada-led-par30-e27-2700k-biv-9-5w-lpar30-9-570wmvs---philips/p</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -7746,20 +8074,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D182" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E182" s="3" t="n"/>
+      <c r="D182" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E182" s="3" t="n">
+        <v>83.31999999999999</v>
+      </c>
       <c r="F182" s="3" t="n"/>
-      <c r="G182" s="2" t="n"/>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H182" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I182" s="2" t="n"/>
-      <c r="J182" s="2" t="inlineStr"/>
-      <c r="K182" s="2" t="inlineStr"/>
+      <c r="J182" s="2" t="inlineStr">
+        <is>
+          <t>Refletor LED Ledvance 10W IP65</t>
+        </is>
+      </c>
+      <c r="K182" s="2" t="inlineStr">
+        <is>
+          <t>Dimensional (SP): https://www.dimensional.com.br/projetor-pt-10w-110-240v-3000k-7016867-ledvance/p | marca premium; genérico sai por ~R$ 20</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
@@ -7777,20 +8119,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D183" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E183" s="3" t="n"/>
+      <c r="D183" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E183" s="3" t="n">
+        <v>62.99</v>
+      </c>
       <c r="F183" s="3" t="n"/>
-      <c r="G183" s="2" t="n"/>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H183" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I183" s="2" t="n"/>
-      <c r="J183" s="2" t="inlineStr"/>
-      <c r="K183" s="2" t="inlineStr"/>
+      <c r="J183" s="2" t="inlineStr">
+        <is>
+          <t>Refletor LED Ledvance 20W IP65</t>
+        </is>
+      </c>
+      <c r="K183" s="2" t="inlineStr">
+        <is>
+          <t>Dimensional (SP): https://www.dimensional.com.br/projetor-led-al-br-sob-ip65-20w-100-240v-3000k-7016880-ledvance/p</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -7808,20 +8164,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D184" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E184" s="3" t="n"/>
+      <c r="D184" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E184" s="3" t="n">
+        <v>79.98999999999999</v>
+      </c>
       <c r="F184" s="3" t="n"/>
-      <c r="G184" s="2" t="n"/>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H184" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I184" s="2" t="n"/>
-      <c r="J184" s="2" t="inlineStr"/>
-      <c r="K184" s="2" t="inlineStr"/>
+      <c r="J184" s="2" t="inlineStr">
+        <is>
+          <t>Refletor LED Ledvance 30W IP65</t>
+        </is>
+      </c>
+      <c r="K184" s="2" t="inlineStr">
+        <is>
+          <t>Dimensional (SP): https://www.dimensional.com.br/projetor-led-al-br-ip65-30w-110-240v-5000k-7016884-ledvance/p</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
@@ -7839,20 +8209,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D185" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E185" s="3" t="n"/>
+      <c r="D185" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E185" s="3" t="n">
+        <v>75.90000000000001</v>
+      </c>
       <c r="F185" s="3" t="n"/>
-      <c r="G185" s="2" t="n"/>
+      <c r="G185" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H185" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I185" s="2" t="n"/>
-      <c r="J185" s="2" t="inlineStr"/>
-      <c r="K185" s="2" t="inlineStr"/>
+      <c r="J185" s="2" t="inlineStr">
+        <is>
+          <t>Balizador LED de solo 1W IP67 Nordecor (2W indisponível)</t>
+        </is>
+      </c>
+      <c r="K185" s="2" t="inlineStr">
+        <is>
+          <t>Leroy Merlin: https://www.leroymerlin.com.br/balizador-led-embutido-de-solo-3000k-bivolt-ip67-nordecor_1570461348</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -7870,20 +8254,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D186" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E186" s="3" t="n"/>
+      <c r="D186" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E186" s="3" t="n">
+        <v>47.9</v>
+      </c>
       <c r="F186" s="3" t="n"/>
-      <c r="G186" s="2" t="n"/>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H186" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I186" s="2" t="n"/>
-      <c r="J186" s="2" t="inlineStr"/>
-      <c r="K186" s="2" t="inlineStr"/>
+      <c r="J186" s="2" t="inlineStr">
+        <is>
+          <t>Balizador LED de solo 5W IP67 Embu Led (6W indisponível)</t>
+        </is>
+      </c>
+      <c r="K186" s="2" t="inlineStr">
+        <is>
+          <t>Leroy Merlin: https://www.leroymerlin.com.br/spot-balizador-de-embutir-piso-solo-ip67-led-5w-3000k-bivolt_1572261743</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
@@ -9496,7 +9894,7 @@
       </c>
       <c r="K225" s="2" t="inlineStr">
         <is>
-          <t>preço herdado de 'Equipamentos e Sistemas - Boiler Baixa Pressão 500 L' por similaridade (0.62)</t>
+          <t>preço herdado de 'Equipamentos e Sistemas - Boiler Baixa Pressão 500 L' por similaridade (0.62) — conferir</t>
         </is>
       </c>
     </row>
@@ -10615,7 +11013,7 @@
       </c>
       <c r="K252" s="2" t="inlineStr">
         <is>
-          <t>preço herdado de 'Fechaduras - Inox Home iX60 (55mm) Interna Black - STAM' por similaridade (0.78)</t>
+          <t>preço herdado de 'Fechaduras - Inox Home iX60 (55mm) Interna Black - STAM' por similaridade (0.78) — conferir</t>
         </is>
       </c>
     </row>
@@ -12906,20 +13304,34 @@
           <t>Locação Ferramentas</t>
         </is>
       </c>
-      <c r="D308" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E308" s="3" t="n"/>
+      <c r="D308" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E308" s="3" t="n">
+        <v>1909</v>
+      </c>
       <c r="F308" s="3" t="n"/>
-      <c r="G308" s="2" t="n"/>
+      <c r="G308" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H308" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I308" s="2" t="n"/>
-      <c r="J308" s="2" t="inlineStr"/>
-      <c r="K308" s="2" t="inlineStr"/>
+      <c r="J308" s="2" t="inlineStr">
+        <is>
+          <t>COMPRA de autotransformador trifásico 5 kVA 220/380V (ABC Transformadores, Diadema/SP) — locadoras de SP só cotam sob consulta</t>
+        </is>
+      </c>
+      <c r="K308" s="2" t="inlineStr">
+        <is>
+          <t>ABC Transformadores (SP): https://www.abctrafos.com.br/auto-transformador-5-kva-220v-380v-trifasico-a-seco-5000-va-reversivel | é preço de compra, não de locação — ajustar quando tiver cotação de locação</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
@@ -14745,7 +15157,7 @@
       </c>
       <c r="K352" s="2" t="inlineStr">
         <is>
-          <t>preço herdado de 'Madeira Estrutura - Tábuas Cedrinho Mescaldo de 30cm x 1,5mts' por similaridade (0.8)</t>
+          <t>preço herdado de 'Madeira Estrutura - Tábuas Cedrinho Mescaldo de 30cm x 1,5mts' por similaridade (0.8) — conferir</t>
         </is>
       </c>
     </row>
@@ -15741,7 +16153,7 @@
       </c>
       <c r="K376" s="2" t="inlineStr">
         <is>
-          <t>preço herdado de 'Metal - Hidráulica - Monocomando de piso Banheira' por similaridade (0.71)</t>
+          <t>preço herdado de 'Metal - Hidráulica - Monocomando de piso Banheira' por similaridade (0.71) — conferir</t>
         </is>
       </c>
     </row>
@@ -18016,7 +18428,7 @@
       </c>
       <c r="K431" s="2" t="inlineStr">
         <is>
-          <t>preço herdado de 'PVC -  Esgoto - Ralo Oculto Quadrado 6''' por similaridade (0.83)</t>
+          <t>preço herdado de 'PVC -  Esgoto - Ralo Oculto Quadrado 6''' por similaridade (0.83) — conferir</t>
         </is>
       </c>
     </row>
@@ -21853,20 +22265,34 @@
           <t>Tubulação PVC</t>
         </is>
       </c>
-      <c r="D525" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E525" s="3" t="n"/>
+      <c r="D525" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E525" s="3" t="n">
+        <v>1.89</v>
+      </c>
       <c r="F525" s="3" t="n"/>
-      <c r="G525" s="2" t="n"/>
+      <c r="G525" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H525" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I525" s="2" t="n"/>
-      <c r="J525" s="2" t="inlineStr"/>
-      <c r="K525" s="2" t="inlineStr"/>
+      <c r="J525" s="2" t="inlineStr">
+        <is>
+          <t>Anel de borracha para esgoto 40 mm Tigre</t>
+        </is>
+      </c>
+      <c r="K525" s="2" t="inlineStr">
+        <is>
+          <t>Telhanorte: https://www.telhanorte.com.br/anel-de-borracha-para-esgoto-adaptador-joelho-40mm-tigre-22748/p</t>
+        </is>
+      </c>
     </row>
     <row r="526">
       <c r="A526" s="2" t="inlineStr">
@@ -22212,20 +22638,34 @@
           <t>Tubulação PVC</t>
         </is>
       </c>
-      <c r="D534" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E534" s="3" t="n"/>
+      <c r="D534" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E534" s="3" t="n">
+        <v>236.9</v>
+      </c>
       <c r="F534" s="3" t="n"/>
-      <c r="G534" s="2" t="n"/>
+      <c r="G534" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H534" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I534" s="2" t="n"/>
-      <c r="J534" s="2" t="inlineStr"/>
-      <c r="K534" s="2" t="inlineStr"/>
+      <c r="J534" s="2" t="inlineStr">
+        <is>
+          <t>Caixa de inspeção de concreto pré-moldada 60x60 cm Concrebox</t>
+        </is>
+      </c>
+      <c r="K534" s="2" t="inlineStr">
+        <is>
+          <t>Telhanorte: https://www.telhanorte.com.br/caixa-de-inspecao-do-ramal-60x60cm-i6-concrebox-1415476/p | composição SINAPI-SP 97906 em alvenaria com mão de obra: R$ 525,39</t>
+        </is>
+      </c>
     </row>
     <row r="535">
       <c r="A535" s="2" t="inlineStr">
@@ -26466,7 +26906,7 @@
       </c>
       <c r="K637" s="2" t="inlineStr">
         <is>
-          <t>preço herdado de 'PVC – Elétrica - Caixa 4x4” pvc embutir' por similaridade (0.83)</t>
+          <t>preço herdado de 'PVC – Elétrica - Caixa 4x4” pvc embutir' por similaridade (0.83) — conferir</t>
         </is>
       </c>
     </row>
@@ -26486,20 +26926,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D638" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E638" s="3" t="n"/>
+      <c r="D638" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E638" s="3" t="n">
+        <v>5.2</v>
+      </c>
       <c r="F638" s="3" t="n"/>
-      <c r="G638" s="2" t="n"/>
+      <c r="G638" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H638" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I638" s="2" t="n"/>
-      <c r="J638" s="2" t="inlineStr"/>
-      <c r="K638" s="2" t="inlineStr"/>
+      <c r="J638" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP insumo 12001 — caixa octogonal 4x4 PVC fundo móvel</t>
+        </is>
+      </c>
+      <c r="K638" s="2" t="inlineStr">
+        <is>
+          <t>SINAPI-SP jul/2026: https://buscadorsinapi.com.br/sp/insumo/12001</t>
+        </is>
+      </c>
     </row>
     <row r="639">
       <c r="A639" s="2" t="inlineStr">
@@ -26767,20 +27221,34 @@
           <t>Tubulação PVC</t>
         </is>
       </c>
-      <c r="D645" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E645" s="3" t="n"/>
+      <c r="D645" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E645" s="3" t="n">
+        <v>8.99</v>
+      </c>
       <c r="F645" s="3" t="n"/>
-      <c r="G645" s="2" t="n"/>
+      <c r="G645" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H645" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I645" s="2" t="n"/>
-      <c r="J645" s="2" t="inlineStr"/>
-      <c r="K645" s="2" t="inlineStr"/>
+      <c r="J645" s="2" t="inlineStr">
+        <is>
+          <t>Eletroduto corrugado PEAD 3" DN90 Kanaduto SW Kanaflex, por metro</t>
+        </is>
+      </c>
+      <c r="K645" s="2" t="inlineStr">
+        <is>
+          <t>Dimensional (SP): https://www.dimensional.com.br/eletroduto-flexivel-nao-metalico-duto-corrugado-polietileno-alta-densidade-pead-cinza-3-dn90-kanaduto-sw-kdtsw9050-kanaflex/p | outras lojas: R$ 10,96–12,49/m</t>
+        </is>
+      </c>
     </row>
     <row r="646">
       <c r="A646" s="2" t="inlineStr">
@@ -29512,20 +29980,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D712" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E712" s="3" t="n"/>
+      <c r="D712" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E712" s="3" t="n">
+        <v>48.99</v>
+      </c>
       <c r="F712" s="3" t="n"/>
-      <c r="G712" s="2" t="n"/>
+      <c r="G712" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H712" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I712" s="2" t="n"/>
-      <c r="J712" s="2" t="inlineStr"/>
-      <c r="K712" s="2" t="inlineStr"/>
+      <c r="J712" s="2" t="inlineStr">
+        <is>
+          <t>Caixa de passagem de embutir aço galvanizado 152x152x82 mm Cemar CPE15GALV</t>
+        </is>
+      </c>
+      <c r="K712" s="2" t="inlineStr">
+        <is>
+          <t>Dimensional (SP): https://www.dimensional.com.br/247033-caixa-passagem-emb-ac-galv-bg-152x152x82mm-cpe-cpe15galv-cemar-legrand/p</t>
+        </is>
+      </c>
     </row>
     <row r="713">
       <c r="A713" s="2" t="inlineStr">
@@ -29625,20 +30107,34 @@
           <t>Elétrica e Iluminação</t>
         </is>
       </c>
-      <c r="D715" s="4" t="inlineStr">
-        <is>
-          <t>sem compra</t>
-        </is>
-      </c>
-      <c r="E715" s="3" t="n"/>
+      <c r="D715" s="6" t="inlineStr">
+        <is>
+          <t>mercado SP</t>
+        </is>
+      </c>
+      <c r="E715" s="3" t="n">
+        <v>252.99</v>
+      </c>
       <c r="F715" s="3" t="n"/>
-      <c r="G715" s="2" t="n"/>
+      <c r="G715" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
       <c r="H715" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I715" s="2" t="n"/>
-      <c r="J715" s="2" t="inlineStr"/>
-      <c r="K715" s="2" t="inlineStr"/>
+      <c r="J715" s="2" t="inlineStr">
+        <is>
+          <t>Caixa de passagem aço galvanizado 402x402x152 mm Cemar (versão sobrepor; embutir ~R$ 280 fora de SP)</t>
+        </is>
+      </c>
+      <c r="K715" s="2" t="inlineStr">
+        <is>
+          <t>Dimensional (SP): https://www.dimensional.com.br/247108-caixa-passagem-sob-ac-galv-quad-402x402x152mm-cps-cps40galvcx-cemar-legrand/p</t>
+        </is>
+      </c>
     </row>
     <row r="716">
       <c r="A716" s="2" t="inlineStr">
@@ -30837,7 +31333,7 @@
       </c>
       <c r="K744" s="2" t="inlineStr">
         <is>
-          <t>preço herdado de 'Telhado - Manta Térmica face dupla' por similaridade (0.67)</t>
+          <t>preço herdado de 'Telhado - Manta Térmica face dupla' por similaridade (0.67) — conferir</t>
         </is>
       </c>
     </row>

</xml_diff>